<commit_message>
Sửa báo cáo theo góp ý lần 2: luồng nộp đơn sớm, mức độ kết luận, NĐ 267/2025
- Chương 3: quy trình 8 khâu có luồng sớm từ Khâu 3 sang Khâu 6, nghiệm thu là bước
  kiểm tra; điều kiện chi theo kết quả Khâu 3; sơ đồ, Bảng 3.3, 3.4, thí điểm đồng bộ;
  danh mục số quản lý nội bộ có phân quyền, chỉ công khai dữ liệu được phép.
- Chương 2, Kết luận: thống nhất mức độ kết luận (giả thuyết, chưa xác định được
  xung đột); phép ghép tên tính theo người, người trùng họ tên không gán, ghi là
  phân tích thăm dò trên danh sách năm 2026.
- Chương 1: tách phân loại pháp lý với phân nhóm quản lý; căn cứ xác lập, thời hạn
  theo từng đối tượng; hợp đồng phân biệt theo nội dung quyền; thêm NĐ 267/2025.
- Kiến nghị chỉ nêu vấn đề NĐ 267/2025 chưa nêu rõ; sửa tên tạp chí bài Võ (2025).
- Bảng giải trình có căn cứ góp ý lần 2; thêm điểm chưa đủ minh chứng.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ThGArqDrUUsqC1zG1BQvVL
</commit_message>
<xml_diff>
--- a/Ban_cuoi/Ban_chinh_sua_02-10-2026/Du_lieu_bieu_do_Chuong_2.xlsx
+++ b/Ban_cuoi/Ban_chinh_sua_02-10-2026/Du_lieu_bieu_do_Chuong_2.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="549">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="795" uniqueCount="552">
   <si>
     <t>DỮ LIỆU VÀ BIỂU ĐỒ CHƯƠNG 2 - THỰC TRẠNG QUẢN LÝ QUYỀN SỞ HỮU TRÍ TUỆ TẠI TRƯỜNG ĐẠI HỌC THÀNH ĐÔ</t>
   </si>
@@ -556,10 +556,22 @@
     <t>88 trên 247, Gini 0,829, 10% dẫn đầu 39,3%</t>
   </si>
   <si>
-    <t>87 trên 246 tên, Gini 0,832, 39,7%; độ nhạy bỏ dấu: 103 tên, Gini 0,822</t>
-  </si>
-  <si>
-    <t>scripts/ra_soat/so_khop_tac_gia.py</t>
+    <t>Đơn vị là người: 83 trên 240 người có họ tên duy nhất, 12 người thuộc 6 nhóm trùng họ tên không gán bài; Gini 0,836, 38,3%; độ nhạy bỏ dấu: 99 người, Gini 0,827. Ghi là phân tích thăm dò trên danh sách năm 2026; bỏ nhận định lực lượng nòng cốt mỏng</t>
+  </si>
+  <si>
+    <t>scripts/ra_soat/so_khop_tac_gia.py; trùng họ tên đối chiếu bằng CCCD, ngày sinh ở dạng tổng hợp</t>
+  </si>
+  <si>
+    <t>Bài báo trên một giảng viên năm 2025</t>
+  </si>
+  <si>
+    <t>1,11</t>
+  </si>
+  <si>
+    <t>Giữ 1,11, ghi rõ mẫu số là 145 giảng viên theo danh sách năm 2026</t>
+  </si>
+  <si>
+    <t>Danh sách nhân sự năm 2026</t>
   </si>
   <si>
     <t>Khả năng tính toán tiêu chí</t>
@@ -1592,9 +1604,6 @@
   </si>
   <si>
     <t>Nhân lực quản lý sở hữu trí tuệ</t>
-  </si>
-  <si>
-    <t>Danh sách nhân sự năm 2026</t>
   </si>
   <si>
     <t>Cơ sở dữ liệu tra cứu, hạ tầng kỹ thuật</t>
@@ -7347,7 +7356,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="32.7109375" customWidth="1"/>
@@ -7551,21 +7560,21 @@
         <v>199</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -7719,21 +7728,21 @@
         <v>246</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>207</v>
+        <v>247</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>250</v>
+        <v>211</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -7755,24 +7764,24 @@
         <v>255</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>55</v>
+        <v>256</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>56</v>
+        <v>257</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="4" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>258</v>
+        <v>55</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>259</v>
+        <v>56</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>260</v>
@@ -7822,21 +7831,21 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="4" t="s">
-        <v>189</v>
+        <v>273</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="4" t="s">
-        <v>276</v>
+        <v>193</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>277</v>
@@ -7922,21 +7931,21 @@
       <c r="A43" s="4" t="s">
         <v>300</v>
       </c>
-      <c r="B43" s="4"/>
+      <c r="B43" s="4" t="s">
+        <v>301</v>
+      </c>
       <c r="C43" s="4" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="4" t="s">
-        <v>303</v>
-      </c>
-      <c r="B44" s="4" t="s">
         <v>304</v>
       </c>
+      <c r="B44" s="4"/>
       <c r="C44" s="4" t="s">
         <v>305</v>
       </c>
@@ -7948,24 +7957,38 @@
       <c r="A45" s="4" t="s">
         <v>307</v>
       </c>
-      <c r="B45" s="4"/>
+      <c r="B45" s="4" t="s">
+        <v>308</v>
+      </c>
       <c r="C45" s="4" t="s">
-        <v>308</v>
-      </c>
-      <c r="D45" s="4"/>
+        <v>309</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>310</v>
+      </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="4" t="s">
-        <v>309</v>
-      </c>
-      <c r="B46" s="4" t="s">
-        <v>310</v>
-      </c>
+        <v>311</v>
+      </c>
+      <c r="B46" s="4"/>
       <c r="C46" s="4" t="s">
-        <v>311</v>
-      </c>
-      <c r="D46" s="4" t="s">
         <v>312</v>
+      </c>
+      <c r="D46" s="4"/>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>316</v>
       </c>
     </row>
   </sheetData>
@@ -7986,53 +8009,53 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="3" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>46</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="4" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="B4" s="4">
         <v>2021</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="F4" s="8">
         <v>0</v>
@@ -8043,19 +8066,19 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="4" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="B5" s="4">
         <v>2021</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="F5" s="8">
         <v>0</v>
@@ -8066,19 +8089,19 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="4" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="B6" s="4">
         <v>2021</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="F6" s="8">
         <v>0</v>
@@ -8089,19 +8112,19 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="4" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="B7" s="4">
         <v>2021</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="F7" s="8">
         <v>0</v>
@@ -8112,19 +8135,19 @@
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="4" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="B8" s="4">
         <v>2021</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="F8" s="8">
         <v>0</v>
@@ -8135,19 +8158,19 @@
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="4" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="B9" s="4">
         <v>2021</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="F9" s="8">
         <v>0</v>
@@ -8158,19 +8181,19 @@
     </row>
     <row r="10" spans="1:9">
       <c r="A10" s="4" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="B10" s="4">
         <v>2022</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="F10" s="8">
         <v>0</v>
@@ -8181,19 +8204,19 @@
     </row>
     <row r="11" spans="1:9">
       <c r="A11" s="4" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="B11" s="4">
         <v>2022</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="F11" s="8">
         <v>0</v>
@@ -8204,19 +8227,19 @@
     </row>
     <row r="12" spans="1:9">
       <c r="A12" s="4" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="B12" s="4">
         <v>2022</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="F12" s="8">
         <v>0</v>
@@ -8227,19 +8250,19 @@
     </row>
     <row r="13" spans="1:9">
       <c r="A13" s="4" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="B13" s="4">
         <v>2022</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="F13" s="8">
         <v>0</v>
@@ -8250,19 +8273,19 @@
     </row>
     <row r="14" spans="1:9">
       <c r="A14" s="4" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="B14" s="4">
         <v>2022</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="F14" s="8">
         <v>0</v>
@@ -8273,19 +8296,19 @@
     </row>
     <row r="15" spans="1:9">
       <c r="A15" s="4" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="B15" s="4">
         <v>2022</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="F15" s="8">
         <v>0</v>
@@ -8296,106 +8319,106 @@
     </row>
     <row r="16" spans="1:9">
       <c r="A16" s="4" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="B16" s="4">
         <v>2022</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="F16" s="8">
         <v>5</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="H16" s="4" t="s">
         <v>118</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" s="4" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="B17" s="4">
         <v>2022</v>
       </c>
       <c r="C17" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="E17" s="4" t="s">
         <v>345</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>324</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>341</v>
       </c>
       <c r="F17" s="8">
         <v>29</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="H17" s="4" t="s">
         <v>116</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
     </row>
     <row r="18" spans="1:9">
       <c r="A18" s="4" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="B18" s="4">
         <v>2022</v>
       </c>
       <c r="C18" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="E18" s="4" t="s">
         <v>345</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>324</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>341</v>
       </c>
       <c r="F18" s="8">
         <v>50</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="H18" s="4" t="s">
         <v>117</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
     </row>
     <row r="19" spans="1:9">
       <c r="A19" s="4" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="B19" s="4">
         <v>2022</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="F19" s="8">
         <v>0</v>
@@ -8406,19 +8429,19 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" s="4" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="B20" s="4">
         <v>2023</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="F20" s="8">
         <v>3</v>
@@ -8429,19 +8452,19 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" s="4" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="B21" s="4">
         <v>2023</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="F21" s="8">
         <v>5</v>
@@ -8452,19 +8475,19 @@
     </row>
     <row r="22" spans="1:9">
       <c r="A22" s="4" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="B22" s="4">
         <v>2023</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="F22" s="8">
         <v>3</v>
@@ -8475,19 +8498,19 @@
     </row>
     <row r="23" spans="1:9">
       <c r="A23" s="4" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="B23" s="4">
         <v>2023</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="F23" s="8">
         <v>3</v>
@@ -8498,19 +8521,19 @@
     </row>
     <row r="24" spans="1:9">
       <c r="A24" s="4" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="B24" s="4">
         <v>2023</v>
       </c>
       <c r="C24" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="D24" s="4" t="s">
         <v>332</v>
       </c>
-      <c r="D24" s="4" t="s">
-        <v>328</v>
-      </c>
       <c r="E24" s="4" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="F24" s="8">
         <v>5</v>
@@ -8521,19 +8544,19 @@
     </row>
     <row r="25" spans="1:9">
       <c r="A25" s="4" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="B25" s="4">
         <v>2023</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="F25" s="8">
         <v>1</v>
@@ -8544,164 +8567,164 @@
     </row>
     <row r="26" spans="1:9">
       <c r="A26" s="4" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="B26" s="4">
         <v>2023</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="F26" s="8">
         <v>50</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="H26" s="4" t="s">
         <v>86</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
     </row>
     <row r="27" spans="1:9">
       <c r="A27" s="4" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="B27" s="4">
         <v>2024</v>
       </c>
       <c r="C27" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="E27" s="4" t="s">
         <v>345</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>328</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>341</v>
       </c>
       <c r="F27" s="8">
         <v>58</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="H27" s="4" t="s">
         <v>86</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
     </row>
     <row r="28" spans="1:9">
       <c r="A28" s="4" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B28" s="4">
         <v>2024</v>
       </c>
       <c r="C28" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="E28" s="4" t="s">
         <v>345</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>328</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>341</v>
       </c>
       <c r="F28" s="8">
         <v>43</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="H28" s="4" t="s">
         <v>117</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
     </row>
     <row r="29" spans="1:9">
       <c r="A29" s="4" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="B29" s="4">
         <v>2024</v>
       </c>
       <c r="C29" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="E29" s="4" t="s">
         <v>345</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>328</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>341</v>
       </c>
       <c r="F29" s="8">
         <v>13.25</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="H29" s="4" t="s">
         <v>116</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
     </row>
     <row r="30" spans="1:9">
       <c r="A30" s="4" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="B30" s="4">
         <v>2024</v>
       </c>
       <c r="C30" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="E30" s="4" t="s">
         <v>345</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>324</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>341</v>
       </c>
       <c r="F30" s="8">
         <v>8.5</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="H30" s="4" t="s">
         <v>86</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
     </row>
     <row r="31" spans="1:9">
       <c r="A31" s="4" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="B31" s="4">
         <v>2024</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="F31" s="8">
         <v>3</v>
@@ -8712,19 +8735,19 @@
     </row>
     <row r="32" spans="1:9">
       <c r="A32" s="4" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="B32" s="4">
         <v>2024</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="F32" s="8">
         <v>0</v>
@@ -8735,19 +8758,19 @@
     </row>
     <row r="33" spans="1:9">
       <c r="A33" s="4" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="B33" s="4">
         <v>2024</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="F33" s="8">
         <v>0</v>
@@ -8758,19 +8781,19 @@
     </row>
     <row r="34" spans="1:9">
       <c r="A34" s="4" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="B34" s="4">
         <v>2024</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="F34" s="8">
         <v>0</v>
@@ -8781,19 +8804,19 @@
     </row>
     <row r="35" spans="1:9">
       <c r="A35" s="4" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="B35" s="4">
         <v>2025</v>
       </c>
       <c r="C35" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="D35" s="4" t="s">
         <v>332</v>
       </c>
-      <c r="D35" s="4" t="s">
-        <v>328</v>
-      </c>
       <c r="E35" s="4" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="F35" s="8">
         <v>5</v>
@@ -8804,19 +8827,19 @@
     </row>
     <row r="36" spans="1:9">
       <c r="A36" s="4" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="B36" s="4">
         <v>2025</v>
       </c>
       <c r="C36" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="D36" s="4" t="s">
         <v>332</v>
       </c>
-      <c r="D36" s="4" t="s">
-        <v>328</v>
-      </c>
       <c r="E36" s="4" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="F36" s="8">
         <v>0</v>
@@ -8827,19 +8850,19 @@
     </row>
     <row r="37" spans="1:9">
       <c r="A37" s="4" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="B37" s="4">
         <v>2025</v>
       </c>
       <c r="C37" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="D37" s="4" t="s">
         <v>332</v>
       </c>
-      <c r="D37" s="4" t="s">
-        <v>328</v>
-      </c>
       <c r="E37" s="4" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="F37" s="8">
         <v>0</v>
@@ -8850,19 +8873,19 @@
     </row>
     <row r="38" spans="1:9">
       <c r="A38" s="4" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="B38" s="4">
         <v>2025</v>
       </c>
       <c r="C38" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="D38" s="4" t="s">
         <v>332</v>
       </c>
-      <c r="D38" s="4" t="s">
-        <v>328</v>
-      </c>
       <c r="E38" s="4" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="F38" s="8">
         <v>0</v>
@@ -8873,94 +8896,94 @@
     </row>
     <row r="39" spans="1:9">
       <c r="A39" s="4" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="B39" s="4">
         <v>2025</v>
       </c>
       <c r="C39" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="E39" s="4" t="s">
         <v>345</v>
-      </c>
-      <c r="D39" s="4" t="s">
-        <v>328</v>
-      </c>
-      <c r="E39" s="4" t="s">
-        <v>341</v>
       </c>
       <c r="F39" s="8">
         <v>30</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="H39" s="4" t="s">
         <v>86</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
     </row>
     <row r="40" spans="1:9">
       <c r="A40" s="4" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="B40" s="4">
         <v>2025</v>
       </c>
       <c r="C40" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="E40" s="4" t="s">
         <v>345</v>
-      </c>
-      <c r="D40" s="4" t="s">
-        <v>328</v>
-      </c>
-      <c r="E40" s="4" t="s">
-        <v>341</v>
       </c>
       <c r="F40" s="8">
         <v>30</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="H40" s="4" t="s">
         <v>86</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
     </row>
     <row r="41" spans="1:9">
       <c r="A41" s="4" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="B41" s="4">
         <v>2025</v>
       </c>
       <c r="C41" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E41" s="4" t="s">
         <v>345</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>384</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>341</v>
       </c>
       <c r="F41" s="8">
         <v>80</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="H41" s="4" t="s">
         <v>111</v>
       </c>
       <c r="I41" s="4" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
     </row>
     <row r="42" spans="1:9">
       <c r="E42" s="3" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="F42" s="8">
         <f>SUM(F4:F41)</f>
@@ -8969,7 +8992,7 @@
     </row>
     <row r="44" spans="1:9">
       <c r="A44" s="2" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
     </row>
   </sheetData>
@@ -8991,7 +9014,7 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -8999,25 +9022,25 @@
         <v>104</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>46</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -9025,10 +9048,10 @@
         <v>108</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="D4" s="4">
         <v>2021</v>
@@ -9037,13 +9060,13 @@
         <v>105</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -9051,10 +9074,10 @@
         <v>108</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="D5" s="4">
         <v>2023</v>
@@ -9063,13 +9086,13 @@
         <v>105</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -9077,10 +9100,10 @@
         <v>109</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="D6" s="4">
         <v>2023</v>
@@ -9089,13 +9112,13 @@
         <v>105</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -9103,10 +9126,10 @@
         <v>109</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="D7" s="4">
         <v>2025</v>
@@ -9115,13 +9138,13 @@
         <v>105</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -9129,10 +9152,10 @@
         <v>109</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="D8" s="4">
         <v>2023</v>
@@ -9141,13 +9164,13 @@
         <v>107</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -9155,25 +9178,25 @@
         <v>110</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="D9" s="4">
         <v>2024</v>
       </c>
       <c r="E9" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="F9" s="4" t="s">
         <v>413</v>
       </c>
-      <c r="F9" s="4" t="s">
-        <v>409</v>
-      </c>
       <c r="G9" s="4" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -9181,25 +9204,25 @@
         <v>110</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="D10" s="4">
         <v>2024</v>
       </c>
       <c r="E10" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="F10" s="4" t="s">
         <v>413</v>
       </c>
-      <c r="F10" s="4" t="s">
-        <v>409</v>
-      </c>
       <c r="G10" s="4" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -9207,25 +9230,25 @@
         <v>110</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="D11" s="4">
         <v>2024</v>
       </c>
       <c r="E11" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="F11" s="4" t="s">
         <v>413</v>
       </c>
-      <c r="F11" s="4" t="s">
-        <v>409</v>
-      </c>
       <c r="G11" s="4" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -9233,25 +9256,25 @@
         <v>110</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="D12" s="4">
         <v>2024</v>
       </c>
       <c r="E12" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="F12" s="4" t="s">
         <v>413</v>
       </c>
-      <c r="F12" s="4" t="s">
-        <v>409</v>
-      </c>
       <c r="G12" s="4" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -9259,25 +9282,25 @@
         <v>110</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="D13" s="4">
         <v>2024</v>
       </c>
       <c r="E13" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="F13" s="4" t="s">
         <v>413</v>
       </c>
-      <c r="F13" s="4" t="s">
-        <v>409</v>
-      </c>
       <c r="G13" s="4" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -9285,10 +9308,10 @@
         <v>111</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="D14" s="4">
         <v>2025</v>
@@ -9297,13 +9320,13 @@
         <v>107</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -9311,10 +9334,10 @@
         <v>111</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="D15" s="4">
         <v>2026</v>
@@ -9323,18 +9346,18 @@
         <v>107</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="2" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
     </row>
   </sheetData>
@@ -9352,160 +9375,160 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="3" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="4" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="4" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="4" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="4" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="4" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="4" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>464</v>
+        <v>468</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="4" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="4" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
     </row>
   </sheetData>
@@ -9525,41 +9548,41 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="3" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>130</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="4" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>135</v>
@@ -9577,15 +9600,15 @@
         <v>52</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="4" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>135</v>
@@ -9603,15 +9626,15 @@
         <v>6</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="4" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>135</v>
@@ -9629,15 +9652,15 @@
         <v>74</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="4" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>493</v>
+        <v>497</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>135</v>
@@ -9655,15 +9678,15 @@
         <v>109</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>494</v>
+        <v>498</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="4" t="s">
-        <v>495</v>
+        <v>499</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>140</v>
@@ -9681,15 +9704,15 @@
         <v>2</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="4" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>140</v>
@@ -9707,15 +9730,15 @@
         <v>7</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="4" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>135</v>
@@ -9733,15 +9756,15 @@
         <v>5</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="4" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>140</v>
@@ -9759,15 +9782,15 @@
         <v>11</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="4" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>508</v>
+        <v>512</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>145</v>
@@ -9785,15 +9808,15 @@
         <v>0</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="4" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>145</v>
@@ -9805,18 +9828,18 @@
         <v>2</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="2" t="s">
-        <v>513</v>
+        <v>517</v>
       </c>
     </row>
   </sheetData>
@@ -9837,7 +9860,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -9845,13 +9868,13 @@
         <v>130</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>515</v>
+        <v>519</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>516</v>
+        <v>520</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -9859,13 +9882,13 @@
         <v>98</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>518</v>
+        <v>522</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>96</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -9873,13 +9896,13 @@
         <v>98</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>520</v>
+        <v>524</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>95</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>521</v>
+        <v>180</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -9887,13 +9910,13 @@
         <v>98</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>97</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -9901,13 +9924,13 @@
         <v>99</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>95</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -9915,13 +9938,13 @@
         <v>99</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>97</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -9929,13 +9952,13 @@
         <v>99</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>96</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -9943,13 +9966,13 @@
         <v>99</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>97</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -9957,13 +9980,13 @@
         <v>100</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>95</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -9971,13 +9994,13 @@
         <v>100</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>96</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -9985,13 +10008,13 @@
         <v>100</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>95</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -9999,13 +10022,13 @@
         <v>100</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>96</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -10013,13 +10036,13 @@
         <v>101</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>96</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -10027,13 +10050,13 @@
         <v>101</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>97</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -10041,13 +10064,13 @@
         <v>101</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>97</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -10055,13 +10078,13 @@
         <v>101</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>97</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -10069,13 +10092,13 @@
         <v>101</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>97</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
     </row>
   </sheetData>

</xml_diff>